<commit_message>
experiments(kkt): CO2 용접기 대여 단가 반영
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014v4o941zghHSMa9tRzfaqP
</commit_message>
<xml_diff>
--- a/experiments/2026-10-12-kkt-drying-furnace-base/estimate/견적서_금강변압기_진공건조로_회전안착_용접_v2.xlsx
+++ b/experiments/2026-10-12-kkt-drying-furnace-base/estimate/견적서_금강변압기_진공건조로_회전안착_용접_v2.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="136">
   <si>
     <t xml:space="preserve">견      적      서</t>
   </si>
@@ -2312,6 +2312,138 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">장비 대여</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">CO2 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">용접기</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">대</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">일</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">대 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">× 3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">일</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">대당 일 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">40</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">만 원</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">장비사용료</t>
   </si>
   <si>
@@ -2322,6 +2454,472 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
+      <t xml:space="preserve">그라인더</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">환기</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">조명</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">재료비</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">CO2 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">가스</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">와이어</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">디스크</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">비파괴검사</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PT/UT</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">요구 시</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">범위 확인 필요</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">방청</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">도장 보수</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">용접부</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">  작업 내용</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">사다리형 일체 베이스 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10,000×5,000×H800 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">제작</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">설치 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(4</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">명 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">× 3</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">일</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">제작작업</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">강재 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">H-250·H-200·H-150·H-125</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">KG</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">자재산출 시트</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">손실 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5% </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">포함</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">제작 기공</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">명 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">× 3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">일</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">방청 도장</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">프라이머 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">회</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">㎡</t>
+  </si>
+  <si>
+    <t xml:space="preserve">자재산출 시트 도장면적</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
       <t xml:space="preserve">용접기</t>
     </r>
     <r>
@@ -2341,7 +2939,21 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">그라인더</t>
+      <t xml:space="preserve">절단기</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">소모품</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">용접봉</t>
     </r>
     <r>
       <rPr>
@@ -2360,21 +2972,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">환기</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">재료비</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">용접봉</t>
+      <t xml:space="preserve">가스</t>
     </r>
     <r>
       <rPr>
@@ -2393,415 +2991,8 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">가스</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">·</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
       <t xml:space="preserve">디스크</t>
     </r>
-  </si>
-  <si>
-    <t xml:space="preserve">비파괴검사</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PT/UT</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">요구 시</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">범위 확인 필요</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">방청</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">·</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">도장 보수</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">용접부</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">  작업 내용</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">: </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">사다리형 일체 베이스 </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10,000×5,000×H800 </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">제작</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">·</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">설치 </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(4</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">명 </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">× 3</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">일</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">제작작업</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">강재 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">H-250·H-200·H-150·H-125</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">KG</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">자재산출 시트</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">손실 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">5% </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">포함</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">제작 기공</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">4</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">명 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">× 3</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">일</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">방청 도장</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">프라이머 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">회</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">㎡</t>
-  </si>
-  <si>
-    <t xml:space="preserve">자재산출 시트 도장면적</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">용접기</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">·</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">절단기</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">소모품</t>
   </si>
   <si>
     <t xml:space="preserve">슬라이딩면 처리</t>
@@ -4350,7 +4541,7 @@
         <v>1</v>
       </c>
       <c r="G13" s="12" t="n">
-        <f aca="false">용접!H24</f>
+        <f aca="false">용접!H25</f>
         <v>25000000</v>
       </c>
       <c r="H13" s="13" t="n">
@@ -5006,7 +5197,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8.4"/>
@@ -5252,45 +5443,47 @@
       <c r="C16" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="D16" s="11" t="s">
+      <c r="D16" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="E16" s="10" t="s">
-        <v>51</v>
+      <c r="E16" s="11" t="s">
+        <v>80</v>
       </c>
       <c r="F16" s="21" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="G16" s="22" t="n">
-        <v>2500000</v>
+        <v>400000</v>
       </c>
       <c r="H16" s="13" t="n">
         <f aca="false">F16*G16</f>
-        <v>2500000</v>
-      </c>
-      <c r="I16" s="23"/>
+        <v>3600000</v>
+      </c>
+      <c r="I16" s="14" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="11"/>
       <c r="B17" s="11"/>
       <c r="C17" s="11" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>81</v>
-      </c>
-      <c r="E17" s="11" t="s">
-        <v>17</v>
+        <v>83</v>
+      </c>
+      <c r="E17" s="10" t="s">
+        <v>51</v>
       </c>
       <c r="F17" s="21" t="n">
         <v>1</v>
       </c>
       <c r="G17" s="22" t="n">
-        <v>3000000</v>
+        <v>800000</v>
       </c>
       <c r="H17" s="13" t="n">
         <f aca="false">F17*G17</f>
-        <v>3000000</v>
+        <v>800000</v>
       </c>
       <c r="I17" s="23"/>
     </row>
@@ -5298,10 +5491,10 @@
       <c r="A18" s="11"/>
       <c r="B18" s="11"/>
       <c r="C18" s="11" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="E18" s="11" t="s">
         <v>17</v>
@@ -5310,24 +5503,22 @@
         <v>1</v>
       </c>
       <c r="G18" s="22" t="n">
-        <v>2500000</v>
+        <v>3000000</v>
       </c>
       <c r="H18" s="13" t="n">
         <f aca="false">F18*G18</f>
-        <v>2500000</v>
-      </c>
-      <c r="I18" s="23" t="s">
-        <v>84</v>
-      </c>
+        <v>3000000</v>
+      </c>
+      <c r="I18" s="23"/>
     </row>
     <row r="19" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="11"/>
       <c r="B19" s="11"/>
       <c r="C19" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="D19" s="11" t="s">
         <v>86</v>
+      </c>
+      <c r="D19" s="10" t="s">
+        <v>87</v>
       </c>
       <c r="E19" s="11" t="s">
         <v>17</v>
@@ -5336,134 +5527,147 @@
         <v>1</v>
       </c>
       <c r="G19" s="22" t="n">
-        <v>1500000</v>
+        <v>2500000</v>
       </c>
       <c r="H19" s="13" t="n">
         <f aca="false">F19*G19</f>
-        <v>1500000</v>
-      </c>
-      <c r="I19" s="23"/>
+        <v>2500000</v>
+      </c>
+      <c r="I19" s="23" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="11" t="s">
-        <v>57</v>
-      </c>
+      <c r="A20" s="11"/>
       <c r="B20" s="11"/>
       <c r="C20" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="D20" s="11"/>
-      <c r="E20" s="10" t="s">
-        <v>56</v>
+        <v>89</v>
+      </c>
+      <c r="D20" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="E20" s="11" t="s">
+        <v>17</v>
       </c>
       <c r="F20" s="21" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G20" s="22" t="n">
-        <v>600000</v>
+        <v>1500000</v>
       </c>
       <c r="H20" s="13" t="n">
         <f aca="false">F20*G20</f>
-        <v>3000000</v>
+        <v>1500000</v>
       </c>
       <c r="I20" s="23"/>
     </row>
     <row r="21" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="11"/>
+      <c r="A21" s="11" t="s">
+        <v>57</v>
+      </c>
       <c r="B21" s="11"/>
       <c r="C21" s="11" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="D21" s="11"/>
       <c r="E21" s="10" t="s">
-        <v>60</v>
-      </c>
-      <c r="F21" s="24" t="n">
-        <v>3.3</v>
-      </c>
-      <c r="G21" s="13"/>
+        <v>56</v>
+      </c>
+      <c r="F21" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="G21" s="22" t="n">
+        <v>600000</v>
+      </c>
       <c r="H21" s="13" t="n">
-        <f aca="false">(H11+H12+H13+H14+H15)*0.033</f>
-        <v>308550</v>
-      </c>
-      <c r="I21" s="23" t="s">
-        <v>61</v>
-      </c>
+        <f aca="false">F21*G21</f>
+        <v>3000000</v>
+      </c>
+      <c r="I21" s="23"/>
     </row>
     <row r="22" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="11"/>
       <c r="B22" s="11"/>
       <c r="C22" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="D22" s="11"/>
+      <c r="E22" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="F22" s="24" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="G22" s="13"/>
+      <c r="H22" s="13" t="n">
+        <f aca="false">(H11+H12+H13+H14+H15)*0.033</f>
+        <v>308550</v>
+      </c>
+      <c r="I22" s="23" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="11"/>
+      <c r="B23" s="11"/>
+      <c r="C23" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="D22" s="11"/>
-      <c r="E22" s="11" t="s">
+      <c r="D23" s="11"/>
+      <c r="E23" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="F22" s="21" t="n">
+      <c r="F23" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="G22" s="22" t="n">
-        <v>2841450</v>
-      </c>
-      <c r="H22" s="13" t="n">
-        <f aca="false">F22*G22</f>
-        <v>2841450</v>
-      </c>
-      <c r="I22" s="23" t="s">
+      <c r="G23" s="22" t="n">
+        <v>941450</v>
+      </c>
+      <c r="H23" s="13" t="n">
+        <f aca="false">F23*G23</f>
+        <v>941450</v>
+      </c>
+      <c r="I23" s="23" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="18"/>
-      <c r="B23" s="18"/>
-      <c r="C23" s="9" t="s">
+    <row r="24" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="18"/>
+      <c r="B24" s="18"/>
+      <c r="C24" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="D23" s="18"/>
-      <c r="E23" s="18"/>
-      <c r="F23" s="25"/>
-      <c r="G23" s="19"/>
-      <c r="H23" s="16" t="n">
-        <f aca="false">SUM(H11:H22)</f>
+      <c r="D24" s="18"/>
+      <c r="E24" s="18"/>
+      <c r="F24" s="25"/>
+      <c r="G24" s="19"/>
+      <c r="H24" s="16" t="n">
+        <f aca="false">SUM(H11:H23)</f>
         <v>25000000</v>
       </c>
-      <c r="I23" s="17"/>
-    </row>
-    <row r="24" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="9" t="s">
+      <c r="I24" s="17"/>
+    </row>
+    <row r="25" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="B24" s="9"/>
-      <c r="C24" s="9"/>
-      <c r="D24" s="9"/>
-      <c r="E24" s="15" t="s">
+      <c r="B25" s="9"/>
+      <c r="C25" s="9"/>
+      <c r="D25" s="9"/>
+      <c r="E25" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="F24" s="15"/>
-      <c r="G24" s="15"/>
-      <c r="H24" s="16" t="n">
-        <f aca="false">H23</f>
+      <c r="F25" s="15"/>
+      <c r="G25" s="15"/>
+      <c r="H25" s="16" t="n">
+        <f aca="false">H24</f>
         <v>25000000</v>
       </c>
-      <c r="I24" s="17"/>
-    </row>
-    <row r="26" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="B26" s="20"/>
-      <c r="C26" s="20"/>
-      <c r="D26" s="20"/>
-      <c r="E26" s="20"/>
-      <c r="F26" s="20"/>
-      <c r="G26" s="20"/>
-      <c r="H26" s="20"/>
-      <c r="I26" s="20"/>
+      <c r="I25" s="17"/>
     </row>
     <row r="27" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="20" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B27" s="20"/>
       <c r="C27" s="20"/>
@@ -5476,7 +5680,7 @@
     </row>
     <row r="28" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="20" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B28" s="20"/>
       <c r="C28" s="20"/>
@@ -5487,8 +5691,21 @@
       <c r="H28" s="20"/>
       <c r="I28" s="20"/>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="26" t="s">
+    <row r="29" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="20" t="s">
+        <v>32</v>
+      </c>
+      <c r="B29" s="20"/>
+      <c r="C29" s="20"/>
+      <c r="D29" s="20"/>
+      <c r="E29" s="20"/>
+      <c r="F29" s="20"/>
+      <c r="G29" s="20"/>
+      <c r="H29" s="20"/>
+      <c r="I29" s="20"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="26" t="s">
         <v>65</v>
       </c>
     </row>
@@ -5503,13 +5720,13 @@
     <mergeCell ref="A10:C10"/>
     <mergeCell ref="A11:B12"/>
     <mergeCell ref="A13:B14"/>
-    <mergeCell ref="A15:B19"/>
-    <mergeCell ref="A20:B22"/>
-    <mergeCell ref="A24:D24"/>
-    <mergeCell ref="E24:G24"/>
-    <mergeCell ref="A26:I26"/>
+    <mergeCell ref="A15:B20"/>
+    <mergeCell ref="A21:B23"/>
+    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="E25:G25"/>
     <mergeCell ref="A27:I27"/>
     <mergeCell ref="A28:I28"/>
+    <mergeCell ref="A29:I29"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -5594,7 +5811,7 @@
     </row>
     <row r="8" customFormat="false" ht="17.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B8" s="7"/>
       <c r="C8" s="7"/>
@@ -5632,17 +5849,17 @@
     </row>
     <row r="11" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B11" s="11"/>
       <c r="C11" s="11" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="F11" s="21" t="n">
         <v>3227</v>
@@ -5655,7 +5872,7 @@
         <v>4195100</v>
       </c>
       <c r="I11" s="23" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5665,7 +5882,7 @@
         <v>37</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="E12" s="10" t="s">
         <v>39</v>
@@ -5681,20 +5898,20 @@
         <v>3600000</v>
       </c>
       <c r="I12" s="14" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="11"/>
       <c r="B13" s="11"/>
       <c r="C13" s="11" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F13" s="21" t="n">
         <v>102</v>
@@ -5707,17 +5924,17 @@
         <v>1530000</v>
       </c>
       <c r="I13" s="23" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="11"/>
       <c r="B14" s="11"/>
       <c r="C14" s="11" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="E14" s="10" t="s">
         <v>51</v>
@@ -5738,10 +5955,10 @@
       <c r="A15" s="11"/>
       <c r="B15" s="11"/>
       <c r="C15" s="11" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>81</v>
+        <v>104</v>
       </c>
       <c r="E15" s="11" t="s">
         <v>17</v>
@@ -5762,10 +5979,10 @@
       <c r="A16" s="11"/>
       <c r="B16" s="11"/>
       <c r="C16" s="11" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="E16" s="11" t="s">
         <v>17</v>
@@ -5781,17 +5998,17 @@
         <v>800000</v>
       </c>
       <c r="I16" s="23" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="11"/>
       <c r="B17" s="11"/>
       <c r="C17" s="11" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="E17" s="11" t="s">
         <v>45</v>
@@ -5814,7 +6031,7 @@
       </c>
       <c r="B18" s="11"/>
       <c r="C18" s="11" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="D18" s="11"/>
       <c r="E18" s="11" t="s">
@@ -5831,7 +6048,7 @@
         <v>1500000</v>
       </c>
       <c r="I18" s="23" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6022,56 +6239,56 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="27" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="28" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="B3" s="28" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="D3" s="15" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="E3" s="15" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="F3" s="15" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="G3" s="15" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="H3" s="15" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="I3" s="15" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="J3" s="15" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="K3" s="15" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="L3" s="15" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="M3" s="15" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="29" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="B4" s="29" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="C4" s="30"/>
       <c r="D4" s="30"/>
@@ -6087,10 +6304,10 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="29" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B5" s="29" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="C5" s="31"/>
       <c r="D5" s="31"/>
@@ -6106,10 +6323,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="29" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="B6" s="29" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="C6" s="31"/>
       <c r="D6" s="31"/>
@@ -6125,10 +6342,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="29" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="B7" s="29" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="C7" s="31"/>
       <c r="D7" s="31"/>
@@ -6144,10 +6361,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="29" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="B8" s="29" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="C8" s="31"/>
       <c r="D8" s="31"/>
@@ -6163,7 +6380,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="26" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
experiments(kkt): 베이스 H빔 250×250 구매 견적 반영
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014v4o941zghHSMa9tRzfaqP
</commit_message>
<xml_diff>
--- a/experiments/2026-10-12-kkt-drying-furnace-base/estimate/견적서_금강변압기_진공건조로_회전안착_용접_v2.xlsx
+++ b/experiments/2026-10-12-kkt-drying-furnace-base/estimate/견적서_금강변압기_진공건조로_회전안착_용접_v2.xlsx
@@ -12,7 +12,8 @@
     <sheet name="도비" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="용접" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="베이스" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="공정표" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="베이스자재" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="공정표" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="149">
   <si>
     <t xml:space="preserve">견      적      서</t>
   </si>
@@ -1126,7 +1127,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">베이스 강재는 개략 산출</t>
+      <t xml:space="preserve">베이스 </t>
     </r>
     <r>
       <rPr>
@@ -1136,7 +1137,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">(</t>
+      <t xml:space="preserve">H</t>
     </r>
     <r>
       <rPr>
@@ -1145,7 +1146,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">약 </t>
+      <t xml:space="preserve">빔은 중고품 기준입니다</t>
     </r>
     <r>
       <rPr>
@@ -1155,7 +1156,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">3.2</t>
+      <t xml:space="preserve">. </t>
     </r>
     <r>
       <rPr>
@@ -1164,7 +1165,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">톤</t>
+      <t xml:space="preserve">신품 적용 시 </t>
     </r>
     <r>
       <rPr>
@@ -1174,7 +1175,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">)</t>
+      <t xml:space="preserve">3,997,657</t>
     </r>
     <r>
       <rPr>
@@ -1183,7 +1184,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">이며 구조검토 결과에 따라 변경될 수 있습니다</t>
+      <t xml:space="preserve">원이 추가됩니다</t>
     </r>
     <r>
       <rPr>
@@ -2656,7 +2657,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">사다리형 일체 베이스 </t>
+      <t xml:space="preserve">사다리형 일체 베이스 제작</t>
     </r>
     <r>
       <rPr>
@@ -2667,7 +2668,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">10,000×5,000×H800 </t>
+      <t xml:space="preserve">·</t>
     </r>
     <r>
       <rPr>
@@ -2677,7 +2678,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">제작</t>
+      <t xml:space="preserve">설치</t>
     </r>
     <r>
       <rPr>
@@ -2688,33 +2689,239 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
+      <t xml:space="preserve">, H-250×250 (4</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">명 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">× 3</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">일</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">자재</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">H</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">빔 구매 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">중고</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">H-250×250, 10m 4EA·5m 16EA·0.6m 30EA</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">공급처 견적</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">신품 시 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">13,575,440</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">원</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">운임</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">H</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">빔 운반</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">공급처 견적</t>
+  </si>
+  <si>
+    <t xml:space="preserve">지 게 차</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">자재 하역</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
       <t xml:space="preserve">·</t>
     </r>
     <r>
       <rPr>
-        <b val="true"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">설치 </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(4</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="12"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">조립</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">일</t>
+  </si>
+  <si>
+    <t xml:space="preserve">제작작업</t>
+  </si>
+  <si>
+    <t xml:space="preserve">제작 기공</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
@@ -2723,8 +2930,7 @@
     </r>
     <r>
       <rPr>
-        <b val="true"/>
-        <sz val="12"/>
+        <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="맑은 고딕"/>
         <family val="0"/>
@@ -2734,18 +2940,210 @@
     </r>
     <r>
       <rPr>
-        <b val="true"/>
-        <sz val="12"/>
+        <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">일</t>
     </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="12"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">용접기</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">절단기</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">소모품</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">용접봉</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">가스</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">디스크</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">슬라이딩면 처리</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">그리스</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·PTFE </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">시트</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">밀착 이동용 레일 상면</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">베이스 자재</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: H</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">빔 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">H-250×250×9×14 (</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">공급처 견적</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">부가세 미포함</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="13"/>
         <color rgb="FF000000"/>
         <rFont val="맑은 고딕"/>
         <family val="0"/>
@@ -2755,118 +3153,289 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">제작작업</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">강재 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">H-250·H-200·H-150·H-125</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">KG</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">자재산출 시트</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">손실 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">5% </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">포함</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">제작 기공</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">4</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">명 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">× 3</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">길이</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(m)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">수량</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(EA)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">총 길이</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(m)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">단위중량</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(kg/m)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">중량</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(kg)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">합계</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">금액</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">원</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">kg</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">당</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">원</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">신품</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">중고 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">견적 반영</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">지게차 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
@@ -2874,58 +3443,79 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">방청 도장</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">프라이머 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">회</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">㎡</t>
-  </si>
-  <si>
-    <t xml:space="preserve">자재산출 시트 도장면적</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">용접기</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
+    <t xml:space="preserve">신품 차액</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF555555"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">단위중량 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF555555"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">72.4 kg/m</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF555555"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">는 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF555555"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">KS H-250×250×9×14 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF555555"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">공칭값이에요</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF555555"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF555555"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">수량</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF555555"/>
         <rFont val="맑은 고딕"/>
         <family val="0"/>
         <charset val="1"/>
@@ -2934,185 +3524,22 @@
     </r>
     <r>
       <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">절단기</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">소모품</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">용접봉</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">·</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">가스</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">·</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">디스크</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">슬라이딩면 처리</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">그리스</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">·PTFE </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">시트</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">밀착 이동용 레일 상면</t>
-  </si>
-  <si>
-    <t xml:space="preserve">화 물 차</t>
-  </si>
-  <si>
-    <t xml:space="preserve">운반</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">구조검토</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">·</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">제작도</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">레일</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">·</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">기둥</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">·</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">지반 지지력</t>
+        <sz val="9"/>
+        <color rgb="FF555555"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">금액은 사용자가 받은 공급처 견적이에요</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF555555"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.</t>
     </r>
   </si>
   <si>
@@ -3778,13 +4205,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* \-_-;_-@_-"/>
     <numFmt numFmtId="166" formatCode="#,##0"/>
     <numFmt numFmtId="167" formatCode="#,##0.0"/>
+    <numFmt numFmtId="168" formatCode="General"/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="25">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3919,6 +4347,27 @@
     </font>
     <font>
       <b val="true"/>
+      <sz val="13"/>
+      <color rgb="FF000000"/>
+      <name val="WenQuanYi Zen Hei"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="13"/>
+      <color rgb="FF000000"/>
+      <name val="맑은 고딕"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="WenQuanYi Zen Hei"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b val="true"/>
       <sz val="14"/>
       <color rgb="FF000000"/>
       <name val="WenQuanYi Zen Hei"/>
@@ -4000,7 +4449,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="44">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -4113,6 +4562,58 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -4122,10 +4623,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4568,7 +5065,7 @@
         <v>1</v>
       </c>
       <c r="G14" s="12" t="n">
-        <f aca="false">베이스!H23</f>
+        <f aca="false">베이스!H22</f>
         <v>18000000</v>
       </c>
       <c r="H14" s="13" t="n">
@@ -5743,7 +6240,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8.4"/>
@@ -5852,24 +6349,24 @@
         <v>92</v>
       </c>
       <c r="B11" s="11"/>
-      <c r="C11" s="11" t="s">
-        <v>84</v>
-      </c>
-      <c r="D11" s="11" t="s">
+      <c r="C11" s="10" t="s">
         <v>93</v>
       </c>
-      <c r="E11" s="10" t="s">
+      <c r="D11" s="10" t="s">
         <v>94</v>
       </c>
+      <c r="E11" s="11" t="s">
+        <v>17</v>
+      </c>
       <c r="F11" s="21" t="n">
-        <v>3227</v>
+        <v>1</v>
       </c>
       <c r="G11" s="22" t="n">
-        <v>1300</v>
+        <v>9577783</v>
       </c>
       <c r="H11" s="13" t="n">
         <f aca="false">F11*G11</f>
-        <v>4195100</v>
+        <v>9577783</v>
       </c>
       <c r="I11" s="23" t="s">
         <v>95</v>
@@ -5879,99 +6376,101 @@
       <c r="A12" s="11"/>
       <c r="B12" s="11"/>
       <c r="C12" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="D12" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="E12" s="10" t="s">
-        <v>39</v>
+      <c r="D12" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="E12" s="11" t="s">
+        <v>17</v>
       </c>
       <c r="F12" s="21" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="G12" s="22" t="n">
-        <v>300000</v>
+        <v>160000</v>
       </c>
       <c r="H12" s="13" t="n">
         <f aca="false">F12*G12</f>
-        <v>3600000</v>
-      </c>
-      <c r="I12" s="14" t="s">
-        <v>97</v>
+        <v>160000</v>
+      </c>
+      <c r="I12" s="23" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="11"/>
       <c r="B13" s="11"/>
       <c r="C13" s="11" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F13" s="21" t="n">
-        <v>102</v>
+        <v>2</v>
       </c>
       <c r="G13" s="22" t="n">
-        <v>15000</v>
+        <v>300000</v>
       </c>
       <c r="H13" s="13" t="n">
         <f aca="false">F13*G13</f>
-        <v>1530000</v>
-      </c>
-      <c r="I13" s="23" t="s">
-        <v>101</v>
-      </c>
+        <v>600000</v>
+      </c>
+      <c r="I13" s="23"/>
     </row>
     <row r="14" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="11"/>
+      <c r="A14" s="11" t="s">
+        <v>102</v>
+      </c>
       <c r="B14" s="11"/>
       <c r="C14" s="11" t="s">
-        <v>82</v>
+        <v>37</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="F14" s="21" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="G14" s="22" t="n">
-        <v>1500000</v>
+        <v>300000</v>
       </c>
       <c r="H14" s="13" t="n">
         <f aca="false">F14*G14</f>
-        <v>1500000</v>
-      </c>
-      <c r="I14" s="23"/>
+        <v>3600000</v>
+      </c>
+      <c r="I14" s="14" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11"/>
       <c r="B15" s="11"/>
       <c r="C15" s="11" t="s">
-        <v>103</v>
+        <v>82</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>104</v>
-      </c>
-      <c r="E15" s="11" t="s">
-        <v>17</v>
+        <v>105</v>
+      </c>
+      <c r="E15" s="10" t="s">
+        <v>51</v>
       </c>
       <c r="F15" s="21" t="n">
         <v>1</v>
       </c>
       <c r="G15" s="22" t="n">
-        <v>1500000</v>
+        <v>1000000</v>
       </c>
       <c r="H15" s="13" t="n">
         <f aca="false">F15*G15</f>
-        <v>1500000</v>
+        <v>1000000</v>
       </c>
       <c r="I15" s="23"/>
     </row>
@@ -5979,10 +6478,10 @@
       <c r="A16" s="11"/>
       <c r="B16" s="11"/>
       <c r="C16" s="11" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E16" s="11" t="s">
         <v>17</v>
@@ -5991,15 +6490,13 @@
         <v>1</v>
       </c>
       <c r="G16" s="22" t="n">
-        <v>800000</v>
+        <v>1000000</v>
       </c>
       <c r="H16" s="13" t="n">
         <f aca="false">F16*G16</f>
-        <v>800000</v>
-      </c>
-      <c r="I16" s="23" t="s">
-        <v>107</v>
-      </c>
+        <v>1000000</v>
+      </c>
+      <c r="I16" s="23"/>
     </row>
     <row r="17" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="11"/>
@@ -6011,7 +6508,7 @@
         <v>109</v>
       </c>
       <c r="E17" s="11" t="s">
-        <v>45</v>
+        <v>17</v>
       </c>
       <c r="F17" s="21" t="n">
         <v>1</v>
@@ -6023,7 +6520,9 @@
         <f aca="false">F17*G17</f>
         <v>500000</v>
       </c>
-      <c r="I17" s="23"/>
+      <c r="I17" s="23" t="s">
+        <v>110</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
@@ -6031,131 +6530,120 @@
       </c>
       <c r="B18" s="11"/>
       <c r="C18" s="11" t="s">
-        <v>110</v>
+        <v>55</v>
       </c>
       <c r="D18" s="11"/>
-      <c r="E18" s="11" t="s">
-        <v>17</v>
+      <c r="E18" s="10" t="s">
+        <v>56</v>
       </c>
       <c r="F18" s="21" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G18" s="22" t="n">
-        <v>1500000</v>
+        <v>300000</v>
       </c>
       <c r="H18" s="13" t="n">
         <f aca="false">F18*G18</f>
-        <v>1500000</v>
-      </c>
-      <c r="I18" s="23" t="s">
-        <v>111</v>
-      </c>
+        <v>900000</v>
+      </c>
+      <c r="I18" s="23"/>
     </row>
     <row r="19" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="11"/>
       <c r="B19" s="11"/>
       <c r="C19" s="11" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="D19" s="11"/>
       <c r="E19" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="F19" s="21" t="n">
-        <v>3</v>
-      </c>
-      <c r="G19" s="22" t="n">
-        <v>500000</v>
-      </c>
+        <v>60</v>
+      </c>
+      <c r="F19" s="24" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="G19" s="13"/>
       <c r="H19" s="13" t="n">
-        <f aca="false">F19*G19</f>
-        <v>1500000</v>
-      </c>
-      <c r="I19" s="23"/>
+        <f aca="false">(H14)*0.033</f>
+        <v>118800</v>
+      </c>
+      <c r="I19" s="23" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="11"/>
       <c r="B20" s="11"/>
       <c r="C20" s="11" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="D20" s="11"/>
-      <c r="E20" s="10" t="s">
-        <v>60</v>
-      </c>
-      <c r="F20" s="24" t="n">
-        <v>3.3</v>
-      </c>
-      <c r="G20" s="13"/>
+      <c r="E20" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="F20" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" s="22" t="n">
+        <v>543417</v>
+      </c>
       <c r="H20" s="13" t="n">
-        <f aca="false">(H12)*0.033</f>
-        <v>118800</v>
+        <f aca="false">F20*G20</f>
+        <v>543417</v>
       </c>
       <c r="I20" s="23" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="11"/>
-      <c r="B21" s="11"/>
-      <c r="C21" s="11" t="s">
-        <v>62</v>
-      </c>
-      <c r="D21" s="11"/>
-      <c r="E21" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="F21" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="G21" s="22" t="n">
-        <v>1256100</v>
-      </c>
-      <c r="H21" s="13" t="n">
-        <f aca="false">F21*G21</f>
-        <v>1256100</v>
-      </c>
-      <c r="I21" s="23" t="s">
-        <v>63</v>
-      </c>
+      <c r="A21" s="18"/>
+      <c r="B21" s="18"/>
+      <c r="C21" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="D21" s="18"/>
+      <c r="E21" s="18"/>
+      <c r="F21" s="25"/>
+      <c r="G21" s="19"/>
+      <c r="H21" s="16" t="n">
+        <f aca="false">SUM(H11:H20)</f>
+        <v>18000000</v>
+      </c>
+      <c r="I21" s="17"/>
     </row>
     <row r="22" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="18"/>
-      <c r="B22" s="18"/>
-      <c r="C22" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="D22" s="18"/>
-      <c r="E22" s="18"/>
-      <c r="F22" s="25"/>
-      <c r="G22" s="19"/>
+      <c r="A22" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="B22" s="9"/>
+      <c r="C22" s="9"/>
+      <c r="D22" s="9"/>
+      <c r="E22" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="F22" s="15"/>
+      <c r="G22" s="15"/>
       <c r="H22" s="16" t="n">
-        <f aca="false">SUM(H11:H21)</f>
+        <f aca="false">H21</f>
         <v>18000000</v>
       </c>
       <c r="I22" s="17"/>
     </row>
-    <row r="23" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="B23" s="9"/>
-      <c r="C23" s="9"/>
-      <c r="D23" s="9"/>
-      <c r="E23" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="F23" s="15"/>
-      <c r="G23" s="15"/>
-      <c r="H23" s="16" t="n">
-        <f aca="false">H22</f>
-        <v>18000000</v>
-      </c>
-      <c r="I23" s="17"/>
+    <row r="24" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="20" t="s">
+        <v>30</v>
+      </c>
+      <c r="B24" s="20"/>
+      <c r="C24" s="20"/>
+      <c r="D24" s="20"/>
+      <c r="E24" s="20"/>
+      <c r="F24" s="20"/>
+      <c r="G24" s="20"/>
+      <c r="H24" s="20"/>
+      <c r="I24" s="20"/>
     </row>
     <row r="25" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="20" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B25" s="20"/>
       <c r="C25" s="20"/>
@@ -6168,7 +6656,7 @@
     </row>
     <row r="26" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="20" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B26" s="20"/>
       <c r="C26" s="20"/>
@@ -6179,26 +6667,13 @@
       <c r="H26" s="20"/>
       <c r="I26" s="20"/>
     </row>
-    <row r="27" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="20" t="s">
-        <v>32</v>
-      </c>
-      <c r="B27" s="20"/>
-      <c r="C27" s="20"/>
-      <c r="D27" s="20"/>
-      <c r="E27" s="20"/>
-      <c r="F27" s="20"/>
-      <c r="G27" s="20"/>
-      <c r="H27" s="20"/>
-      <c r="I27" s="20"/>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="26" t="s">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="26" t="s">
         <v>65</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="15">
     <mergeCell ref="A1:I2"/>
     <mergeCell ref="A4:C4"/>
     <mergeCell ref="G4:I4"/>
@@ -6206,13 +6681,14 @@
     <mergeCell ref="G5:I5"/>
     <mergeCell ref="A8:I8"/>
     <mergeCell ref="A10:C10"/>
-    <mergeCell ref="A11:B17"/>
-    <mergeCell ref="A18:B21"/>
-    <mergeCell ref="A23:D23"/>
-    <mergeCell ref="E23:G23"/>
+    <mergeCell ref="A11:B13"/>
+    <mergeCell ref="A14:B17"/>
+    <mergeCell ref="A18:B20"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="E22:G22"/>
+    <mergeCell ref="A24:I24"/>
     <mergeCell ref="A25:I25"/>
     <mergeCell ref="A26:I26"/>
-    <mergeCell ref="A27:I27"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -6229,6 +6705,193 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:E16"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="27" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="28" t="n">
+        <v>10</v>
+      </c>
+      <c r="B4" s="28" t="n">
+        <v>4</v>
+      </c>
+      <c r="C4" s="29" t="n">
+        <f aca="false">A4*B4</f>
+        <v>40</v>
+      </c>
+      <c r="D4" s="28" t="n">
+        <v>72.4</v>
+      </c>
+      <c r="E4" s="30" t="n">
+        <f aca="false">C4*D4</f>
+        <v>2896</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="28" t="n">
+        <v>5</v>
+      </c>
+      <c r="B5" s="28" t="n">
+        <v>16</v>
+      </c>
+      <c r="C5" s="29" t="n">
+        <f aca="false">A5*B5</f>
+        <v>80</v>
+      </c>
+      <c r="D5" s="28" t="n">
+        <v>72.4</v>
+      </c>
+      <c r="E5" s="30" t="n">
+        <f aca="false">C5*D5</f>
+        <v>5792</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="28" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="B6" s="28" t="n">
+        <v>30</v>
+      </c>
+      <c r="C6" s="29" t="n">
+        <f aca="false">A6*B6</f>
+        <v>18</v>
+      </c>
+      <c r="D6" s="28" t="n">
+        <v>72.4</v>
+      </c>
+      <c r="E6" s="30" t="n">
+        <f aca="false">C6*D6</f>
+        <v>1303.2</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="31"/>
+      <c r="B7" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="C7" s="31" t="n">
+        <f aca="false">SUM(C4:C6)</f>
+        <v>138</v>
+      </c>
+      <c r="D7" s="31"/>
+      <c r="E7" s="32" t="n">
+        <f aca="false">SUM(E4:E6)</f>
+        <v>9991.2</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="33" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="33" t="s">
+        <v>118</v>
+      </c>
+      <c r="C9" s="34" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="35" t="s">
+        <v>120</v>
+      </c>
+      <c r="B10" s="36" t="n">
+        <v>13575440</v>
+      </c>
+      <c r="C10" s="37" t="n">
+        <f aca="false">B10/$E$7</f>
+        <v>1358.73969092802</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="35" t="s">
+        <v>121</v>
+      </c>
+      <c r="B11" s="36" t="n">
+        <v>9577783</v>
+      </c>
+      <c r="C11" s="37" t="n">
+        <f aca="false">B11/$E$7</f>
+        <v>958.621887260789</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="35" t="s">
+        <v>96</v>
+      </c>
+      <c r="B12" s="36" t="n">
+        <v>160000</v>
+      </c>
+      <c r="C12" s="35"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="35" t="s">
+        <v>122</v>
+      </c>
+      <c r="B13" s="36" t="n">
+        <v>600000</v>
+      </c>
+      <c r="C13" s="35"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="38" t="s">
+        <v>123</v>
+      </c>
+      <c r="B14" s="39" t="n">
+        <f aca="false">B10-B11</f>
+        <v>3997657</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="26" t="s">
+        <v>124</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:M10"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -6238,149 +6901,149 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="27" t="s">
-        <v>112</v>
+      <c r="A1" s="40" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="28" t="s">
-        <v>113</v>
-      </c>
-      <c r="B3" s="28" t="s">
-        <v>114</v>
+      <c r="A3" s="41" t="s">
+        <v>126</v>
+      </c>
+      <c r="B3" s="41" t="s">
+        <v>127</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>115</v>
+        <v>128</v>
       </c>
       <c r="D3" s="15" t="s">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="E3" s="15" t="s">
-        <v>117</v>
+        <v>130</v>
       </c>
       <c r="F3" s="15" t="s">
-        <v>118</v>
+        <v>131</v>
       </c>
       <c r="G3" s="15" t="s">
-        <v>119</v>
+        <v>132</v>
       </c>
       <c r="H3" s="15" t="s">
-        <v>120</v>
+        <v>133</v>
       </c>
       <c r="I3" s="15" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="J3" s="15" t="s">
-        <v>122</v>
+        <v>135</v>
       </c>
       <c r="K3" s="15" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
       <c r="L3" s="15" t="s">
-        <v>124</v>
+        <v>137</v>
       </c>
       <c r="M3" s="15" t="s">
-        <v>125</v>
+        <v>138</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="29" t="s">
-        <v>126</v>
-      </c>
-      <c r="B4" s="29" t="s">
-        <v>127</v>
-      </c>
-      <c r="C4" s="30"/>
-      <c r="D4" s="30"/>
-      <c r="E4" s="30"/>
-      <c r="F4" s="31"/>
-      <c r="G4" s="31"/>
-      <c r="H4" s="31"/>
-      <c r="I4" s="31"/>
-      <c r="J4" s="31"/>
-      <c r="K4" s="31"/>
-      <c r="L4" s="31"/>
-      <c r="M4" s="31"/>
+      <c r="A4" s="42" t="s">
+        <v>139</v>
+      </c>
+      <c r="B4" s="42" t="s">
+        <v>140</v>
+      </c>
+      <c r="C4" s="43"/>
+      <c r="D4" s="43"/>
+      <c r="E4" s="43"/>
+      <c r="F4" s="35"/>
+      <c r="G4" s="35"/>
+      <c r="H4" s="35"/>
+      <c r="I4" s="35"/>
+      <c r="J4" s="35"/>
+      <c r="K4" s="35"/>
+      <c r="L4" s="35"/>
+      <c r="M4" s="35"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="29" t="s">
-        <v>128</v>
-      </c>
-      <c r="B5" s="29" t="s">
-        <v>129</v>
-      </c>
-      <c r="C5" s="31"/>
-      <c r="D5" s="31"/>
-      <c r="E5" s="31"/>
-      <c r="F5" s="30"/>
-      <c r="G5" s="31"/>
-      <c r="H5" s="31"/>
-      <c r="I5" s="31"/>
-      <c r="J5" s="31"/>
-      <c r="K5" s="31"/>
-      <c r="L5" s="31"/>
-      <c r="M5" s="31"/>
+      <c r="A5" s="42" t="s">
+        <v>141</v>
+      </c>
+      <c r="B5" s="42" t="s">
+        <v>142</v>
+      </c>
+      <c r="C5" s="35"/>
+      <c r="D5" s="35"/>
+      <c r="E5" s="35"/>
+      <c r="F5" s="43"/>
+      <c r="G5" s="35"/>
+      <c r="H5" s="35"/>
+      <c r="I5" s="35"/>
+      <c r="J5" s="35"/>
+      <c r="K5" s="35"/>
+      <c r="L5" s="35"/>
+      <c r="M5" s="35"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="29" t="s">
-        <v>130</v>
-      </c>
-      <c r="B6" s="29" t="s">
-        <v>131</v>
-      </c>
-      <c r="C6" s="31"/>
-      <c r="D6" s="31"/>
-      <c r="E6" s="31"/>
-      <c r="F6" s="31"/>
-      <c r="G6" s="30"/>
-      <c r="H6" s="30"/>
-      <c r="I6" s="31"/>
-      <c r="J6" s="31"/>
-      <c r="K6" s="31"/>
-      <c r="L6" s="31"/>
-      <c r="M6" s="31"/>
+      <c r="A6" s="42" t="s">
+        <v>143</v>
+      </c>
+      <c r="B6" s="42" t="s">
+        <v>144</v>
+      </c>
+      <c r="C6" s="35"/>
+      <c r="D6" s="35"/>
+      <c r="E6" s="35"/>
+      <c r="F6" s="35"/>
+      <c r="G6" s="43"/>
+      <c r="H6" s="43"/>
+      <c r="I6" s="35"/>
+      <c r="J6" s="35"/>
+      <c r="K6" s="35"/>
+      <c r="L6" s="35"/>
+      <c r="M6" s="35"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="29" t="s">
-        <v>132</v>
-      </c>
-      <c r="B7" s="29" t="s">
-        <v>129</v>
-      </c>
-      <c r="C7" s="31"/>
-      <c r="D7" s="31"/>
-      <c r="E7" s="31"/>
-      <c r="F7" s="31"/>
-      <c r="G7" s="31"/>
-      <c r="H7" s="31"/>
-      <c r="I7" s="30"/>
-      <c r="J7" s="30"/>
-      <c r="K7" s="31"/>
-      <c r="L7" s="31"/>
-      <c r="M7" s="31"/>
+      <c r="A7" s="42" t="s">
+        <v>145</v>
+      </c>
+      <c r="B7" s="42" t="s">
+        <v>142</v>
+      </c>
+      <c r="C7" s="35"/>
+      <c r="D7" s="35"/>
+      <c r="E7" s="35"/>
+      <c r="F7" s="35"/>
+      <c r="G7" s="35"/>
+      <c r="H7" s="35"/>
+      <c r="I7" s="43"/>
+      <c r="J7" s="43"/>
+      <c r="K7" s="35"/>
+      <c r="L7" s="35"/>
+      <c r="M7" s="35"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="29" t="s">
-        <v>133</v>
-      </c>
-      <c r="B8" s="29" t="s">
-        <v>134</v>
-      </c>
-      <c r="C8" s="31"/>
-      <c r="D8" s="31"/>
-      <c r="E8" s="31"/>
-      <c r="F8" s="31"/>
-      <c r="G8" s="31"/>
-      <c r="H8" s="31"/>
-      <c r="I8" s="31"/>
-      <c r="J8" s="31"/>
-      <c r="K8" s="30"/>
-      <c r="L8" s="30"/>
-      <c r="M8" s="30"/>
+      <c r="A8" s="42" t="s">
+        <v>146</v>
+      </c>
+      <c r="B8" s="42" t="s">
+        <v>147</v>
+      </c>
+      <c r="C8" s="35"/>
+      <c r="D8" s="35"/>
+      <c r="E8" s="35"/>
+      <c r="F8" s="35"/>
+      <c r="G8" s="35"/>
+      <c r="H8" s="35"/>
+      <c r="I8" s="35"/>
+      <c r="J8" s="35"/>
+      <c r="K8" s="43"/>
+      <c r="L8" s="43"/>
+      <c r="M8" s="43"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="26" t="s">
-        <v>135</v>
+        <v>148</v>
       </c>
     </row>
   </sheetData>

</xml_diff>